<commit_message>
US006(docs): fixed class diagram & updated ReadMe file
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\IdeaProjects\lapr2\docs\sprint2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63eef7978e99d393/Documents/GitHub/sem2-pi24.25-G092-repo/docs/sprint3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FB3E96-C9FB-4BD1-A8A6-997F8E596D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{C4FB3E96-C9FB-4BD1-A8A6-997F8E596D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{208EEB16-1799-4054-B81D-7949A7E6C48D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1566,27 +1566,17 @@
       <c r="C10" s="25">
         <v>1241323</v>
       </c>
-      <c r="D10" s="53">
-        <v>5</v>
-      </c>
-      <c r="E10" s="26">
-        <v>5</v>
-      </c>
-      <c r="F10" s="27">
-        <v>5</v>
-      </c>
-      <c r="G10" s="27">
-        <v>5</v>
-      </c>
-      <c r="H10" s="27">
-        <v>5</v>
-      </c>
+      <c r="D10" s="53"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
       <c r="I10" s="27"/>
       <c r="J10" s="27"/>
       <c r="K10" s="25"/>
-      <c r="L10" s="35">
+      <c r="L10" s="35" t="e">
         <f t="shared" ref="L10:L17" si="0">AVERAGE(D10:K10)</f>
-        <v>5</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1594,27 +1584,17 @@
       <c r="C11" s="6">
         <v>1241176</v>
       </c>
-      <c r="D11" s="7">
-        <v>5</v>
-      </c>
-      <c r="E11" s="53">
-        <v>5</v>
-      </c>
-      <c r="F11" s="24">
-        <v>5</v>
-      </c>
-      <c r="G11" s="6">
-        <v>5</v>
-      </c>
-      <c r="H11" s="6">
-        <v>5</v>
-      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="53"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="36">
+      <c r="L11" s="36" t="e">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1622,27 +1602,17 @@
       <c r="C12" s="6">
         <v>1241166</v>
       </c>
-      <c r="D12" s="6">
-        <v>5</v>
-      </c>
-      <c r="E12" s="7">
-        <v>5</v>
-      </c>
-      <c r="F12" s="53">
-        <v>5</v>
-      </c>
-      <c r="G12" s="24">
-        <v>5</v>
-      </c>
-      <c r="H12" s="6">
-        <v>5</v>
-      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="53"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="8"/>
-      <c r="L12" s="36">
+      <c r="L12" s="36" t="e">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1650,27 +1620,17 @@
       <c r="C13" s="6">
         <v>1241285</v>
       </c>
-      <c r="D13" s="6">
-        <v>5</v>
-      </c>
-      <c r="E13" s="6">
-        <v>5</v>
-      </c>
-      <c r="F13" s="7">
-        <v>5</v>
-      </c>
-      <c r="G13" s="53">
-        <v>5</v>
-      </c>
-      <c r="H13" s="24">
-        <v>5</v>
-      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="53"/>
+      <c r="H13" s="24"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="36">
+      <c r="L13" s="36" t="e">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1678,27 +1638,17 @@
       <c r="C14" s="6">
         <v>1220804</v>
       </c>
-      <c r="D14" s="6">
-        <v>5</v>
-      </c>
-      <c r="E14" s="6">
-        <v>5</v>
-      </c>
-      <c r="F14" s="6">
-        <v>5</v>
-      </c>
-      <c r="G14" s="7">
-        <v>5</v>
-      </c>
-      <c r="H14" s="53">
-        <v>5</v>
-      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="53"/>
       <c r="I14" s="24"/>
       <c r="J14" s="6"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="36">
+      <c r="L14" s="36" t="e">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1760,25 +1710,25 @@
       <c r="C18" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="D18" s="33">
+      <c r="D18" s="33" t="e">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>5</v>
-      </c>
-      <c r="E18" s="33">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E18" s="33" t="e">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="F18" s="33">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F18" s="33" t="e">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="G18" s="33">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G18" s="33" t="e">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="H18" s="33">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H18" s="33" t="e">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -2921,21 +2871,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3119,31 +3054,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3159,4 +3085,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
US003/009(docs): added split diagrams
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63eef7978e99d393/Documents/GitHub/sem2-pi24.25-G092-repo/docs/sprint3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\IdeaProjects\lapr2\docs\sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{C4FB3E96-C9FB-4BD1-A8A6-997F8E596D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{208EEB16-1799-4054-B81D-7949A7E6C48D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419598E0-7F14-46D6-8D19-584D951A44EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1584,17 +1584,27 @@
       <c r="C11" s="6">
         <v>1241176</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
+      <c r="D11" s="7">
+        <v>3</v>
+      </c>
+      <c r="E11" s="53">
+        <v>5</v>
+      </c>
+      <c r="F11" s="24">
+        <v>5</v>
+      </c>
+      <c r="G11" s="6">
+        <v>3</v>
+      </c>
+      <c r="H11" s="6">
+        <v>4</v>
+      </c>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="36" t="e">
+      <c r="L11" s="36">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1602,17 +1612,27 @@
       <c r="C12" s="6">
         <v>1241166</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="6"/>
+      <c r="D12" s="6">
+        <v>3</v>
+      </c>
+      <c r="E12" s="7">
+        <v>5</v>
+      </c>
+      <c r="F12" s="53">
+        <v>5</v>
+      </c>
+      <c r="G12" s="24">
+        <v>1</v>
+      </c>
+      <c r="H12" s="6">
+        <v>2</v>
+      </c>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="8"/>
-      <c r="L12" s="36" t="e">
+      <c r="L12" s="36">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1638,17 +1658,27 @@
       <c r="C14" s="6">
         <v>1220804</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="53"/>
+      <c r="D14" s="6">
+        <v>3</v>
+      </c>
+      <c r="E14" s="6">
+        <v>5</v>
+      </c>
+      <c r="F14" s="6">
+        <v>5</v>
+      </c>
+      <c r="G14" s="7">
+        <v>2</v>
+      </c>
+      <c r="H14" s="53">
+        <v>4</v>
+      </c>
       <c r="I14" s="24"/>
       <c r="J14" s="6"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="36" t="e">
+      <c r="L14" s="36">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1710,25 +1740,25 @@
       <c r="C18" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="D18" s="33" t="e">
+      <c r="D18" s="33">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E18" s="33" t="e">
+        <v>3</v>
+      </c>
+      <c r="E18" s="33">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F18" s="33" t="e">
+        <v>5</v>
+      </c>
+      <c r="F18" s="33">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G18" s="33" t="e">
+        <v>5</v>
+      </c>
+      <c r="G18" s="33">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H18" s="33" t="e">
+        <v>2</v>
+      </c>
+      <c r="H18" s="33">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -2871,6 +2901,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3054,22 +3099,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3085,28 +3139,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "US005(code): JavaFX fixes"
This reverts commit dd8378720eeed0ca430783f541dd78fd89f191e5.
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcapa\IdeaProjects\sem2-pi24.25-G092-repo\docs\sprint3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaom\OneDrive\Ambiente de Trabalho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A1DE48-73B8-4CB3-9D16-2DB023B56C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1095,7 +1095,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Instructions"/>
@@ -1640,27 +1640,17 @@
       <c r="C13" s="6">
         <v>1241285</v>
       </c>
-      <c r="D13" s="6">
-        <v>5</v>
-      </c>
-      <c r="E13" s="6">
-        <v>3</v>
-      </c>
-      <c r="F13" s="7">
-        <v>4</v>
-      </c>
-      <c r="G13" s="53">
-        <v>4</v>
-      </c>
-      <c r="H13" s="24">
-        <v>3</v>
-      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="53"/>
+      <c r="H13" s="24"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="36">
+      <c r="L13" s="36" t="e">
         <f t="shared" si="0"/>
-        <v>3.8</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -1752,23 +1742,23 @@
       </c>
       <c r="D18" s="33">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>3.75</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="E18" s="33">
         <f t="shared" si="1"/>
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="F18" s="33">
         <f t="shared" si="1"/>
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="G18" s="33">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="H18" s="33">
         <f t="shared" si="1"/>
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -2911,18 +2901,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3110,14 +3100,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -3129,6 +3111,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Reapply "US005(code): JavaFX fixes"
This reverts commit b2d72a0a600a9e671c44113c800422c29f47689e.
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaom\OneDrive\Ambiente de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcapa\IdeaProjects\sem2-pi24.25-G092-repo\docs\sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A1DE48-73B8-4CB3-9D16-2DB023B56C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1095,7 +1095,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Instructions"/>
@@ -1640,17 +1640,27 @@
       <c r="C13" s="6">
         <v>1241285</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="53"/>
-      <c r="H13" s="24"/>
+      <c r="D13" s="6">
+        <v>5</v>
+      </c>
+      <c r="E13" s="6">
+        <v>3</v>
+      </c>
+      <c r="F13" s="7">
+        <v>4</v>
+      </c>
+      <c r="G13" s="53">
+        <v>4</v>
+      </c>
+      <c r="H13" s="24">
+        <v>3</v>
+      </c>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="36" t="e">
+      <c r="L13" s="36">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -1742,23 +1752,23 @@
       </c>
       <c r="D18" s="33">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>3.3333333333333335</v>
+        <v>3.75</v>
       </c>
       <c r="E18" s="33">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="F18" s="33">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="G18" s="33">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H18" s="33">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -2901,18 +2911,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3100,6 +3110,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -3111,14 +3129,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
(code): final additions to project
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcapa\IdeaProjects\sem2-pi24.25-G092-repo\docs\sprint3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63eef7978e99d393/Documents/GitHub/sem2-pi24.25-G092-repo/docs/sprint3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4BD0B80-14EA-488D-8DD4-0E5586C9FE97}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1095,7 +1095,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Instructions"/>
@@ -1464,33 +1464,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6.25" customWidth="1"/>
+    <col min="2" max="2" width="6.19921875" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="12" width="7.875" customWidth="1"/>
+    <col min="4" max="12" width="7.8984375" customWidth="1"/>
     <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1499,13 +1499,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:13" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:13" ht="15.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="E8" s="58" t="s">
@@ -1520,7 +1520,7 @@
       <c r="L8" s="59"/>
       <c r="M8" s="60"/>
     </row>
-    <row r="9" spans="1:13" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="105.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="29">
@@ -1559,33 +1559,43 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="55" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="25">
         <v>1241323</v>
       </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
+      <c r="D10" s="53">
+        <v>5</v>
+      </c>
+      <c r="E10" s="26">
+        <v>5</v>
+      </c>
+      <c r="F10" s="27">
+        <v>5</v>
+      </c>
+      <c r="G10" s="27">
+        <v>4</v>
+      </c>
+      <c r="H10" s="27">
+        <v>4</v>
+      </c>
       <c r="I10" s="27"/>
       <c r="J10" s="27"/>
       <c r="K10" s="25"/>
-      <c r="L10" s="35" t="e">
+      <c r="L10" s="35">
         <f t="shared" ref="L10:L17" si="0">AVERAGE(D10:K10)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="56"/>
       <c r="C11" s="6">
         <v>1241176</v>
       </c>
       <c r="D11" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" s="53">
         <v>5</v>
@@ -1594,7 +1604,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H11" s="6">
         <v>4</v>
@@ -1604,10 +1614,10 @@
       <c r="K11" s="8"/>
       <c r="L11" s="36">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="56"/>
       <c r="C12" s="6">
         <v>1241166</v>
@@ -1635,7 +1645,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="56"/>
       <c r="C13" s="6">
         <v>1241285</v>
@@ -1663,13 +1673,13 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="56"/>
       <c r="C14" s="6">
         <v>1220804</v>
       </c>
       <c r="D14" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" s="6">
         <v>5</v>
@@ -1678,7 +1688,7 @@
         <v>5</v>
       </c>
       <c r="G14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="53">
         <v>4</v>
@@ -1691,7 +1701,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="56"/>
       <c r="C15" s="6" t="s">
         <v>6</v>
@@ -1709,7 +1719,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="56"/>
       <c r="C16" s="6" t="s">
         <v>7</v>
@@ -1727,7 +1737,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="57"/>
       <c r="C17" s="28" t="s">
         <v>8</v>
@@ -1745,30 +1755,30 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="1"/>
       <c r="C18" s="32" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="33">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>3.75</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E18" s="33">
         <f t="shared" si="1"/>
-        <v>4.5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="F18" s="33">
         <f t="shared" si="1"/>
-        <v>4.75</v>
+        <v>4.8</v>
       </c>
       <c r="G18" s="33">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="H18" s="33">
         <f t="shared" si="1"/>
-        <v>3.75</v>
+        <v>3.8</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -1784,7 +1794,7 @@
       </c>
       <c r="L18" s="38"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="42" t="s">
         <v>9</v>
       </c>
@@ -1800,7 +1810,7 @@
       <c r="K20" s="43"/>
       <c r="L20" s="44"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="45" t="s">
         <v>35</v>
       </c>
@@ -1816,7 +1826,7 @@
       <c r="K21" s="46"/>
       <c r="L21" s="47"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="48" t="s">
         <v>36</v>
       </c>
@@ -1832,7 +1842,7 @@
       <c r="K22" s="46"/>
       <c r="L22" s="47"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="45" t="s">
         <v>37</v>
       </c>
@@ -1848,7 +1858,7 @@
       <c r="K23" s="46"/>
       <c r="L23" s="47"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="45"/>
       <c r="B24" s="46"/>
       <c r="C24" s="46"/>
@@ -1862,7 +1872,7 @@
       <c r="K24" s="46"/>
       <c r="L24" s="47"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="49" t="s">
         <v>38</v>
       </c>
@@ -1878,7 +1888,7 @@
       <c r="K25" s="46"/>
       <c r="L25" s="47"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="45">
         <v>0</v>
       </c>
@@ -1896,7 +1906,7 @@
       <c r="K26" s="46"/>
       <c r="L26" s="47"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="45">
         <v>1</v>
       </c>
@@ -1914,7 +1924,7 @@
       <c r="K27" s="46"/>
       <c r="L27" s="47"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="45">
         <v>2</v>
       </c>
@@ -1932,7 +1942,7 @@
       <c r="K28" s="46"/>
       <c r="L28" s="47"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="45">
         <v>3</v>
       </c>
@@ -1950,7 +1960,7 @@
       <c r="K29" s="46"/>
       <c r="L29" s="47"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="45">
         <v>4</v>
       </c>
@@ -1968,7 +1978,7 @@
       <c r="K30" s="46"/>
       <c r="L30" s="47"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="45">
         <v>5</v>
       </c>
@@ -1986,7 +1996,7 @@
       <c r="K31" s="46"/>
       <c r="L31" s="47"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="50"/>
       <c r="B32" s="51"/>
       <c r="C32" s="51"/>
@@ -2019,21 +2029,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="20.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.09765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="10" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="55" t="s">
         <v>17</v>
       </c>
@@ -2065,7 +2075,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A4" s="56"/>
       <c r="B4" s="64"/>
       <c r="C4" s="64"/>
@@ -2089,7 +2099,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="56"/>
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
@@ -2113,7 +2123,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>41</v>
       </c>
@@ -2143,7 +2153,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>42</v>
       </c>
@@ -2173,7 +2183,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>43</v>
       </c>
@@ -2203,7 +2213,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>44</v>
       </c>
@@ -2233,7 +2243,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>45</v>
       </c>
@@ -2263,7 +2273,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>46</v>
       </c>
@@ -2293,7 +2303,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>47</v>
       </c>
@@ -2323,7 +2333,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>48</v>
       </c>
@@ -2353,7 +2363,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>49</v>
       </c>
@@ -2383,7 +2393,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>50</v>
       </c>
@@ -2413,7 +2423,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>51</v>
       </c>
@@ -2443,7 +2453,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>52</v>
       </c>
@@ -2473,7 +2483,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>53</v>
       </c>
@@ -2505,7 +2515,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>54</v>
       </c>
@@ -2535,7 +2545,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>55</v>
       </c>
@@ -2565,7 +2575,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>56</v>
       </c>
@@ -2595,7 +2605,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>57</v>
       </c>
@@ -2625,7 +2635,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>58</v>
       </c>
@@ -2655,7 +2665,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>40</v>
       </c>
@@ -2685,7 +2695,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A25" s="11"/>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -2709,7 +2719,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A26" s="11"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -2733,7 +2743,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A27" s="11"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -2757,7 +2767,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A28" s="11"/>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -2781,7 +2791,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A29" s="11"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -2805,7 +2815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A30" s="11"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -2829,7 +2839,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A31" s="11"/>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -2853,7 +2863,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="15"/>
       <c r="B32" s="39"/>
       <c r="C32" s="18"/>
@@ -2920,12 +2930,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3109,6 +3113,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
   <ds:schemaRefs>
@@ -3118,22 +3128,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3149,4 +3143,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "(code): final additions to project"
This reverts commit e7b31db4d24a580336105bed642af491d3d314f0.
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63eef7978e99d393/Documents/GitHub/sem2-pi24.25-G092-repo/docs/sprint3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcapa\IdeaProjects\sem2-pi24.25-G092-repo\docs\sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4BD0B80-14EA-488D-8DD4-0E5586C9FE97}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1095,7 +1095,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Instructions"/>
@@ -1464,33 +1464,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.19921875" customWidth="1"/>
+    <col min="2" max="2" width="6.25" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="12" width="7.8984375" customWidth="1"/>
+    <col min="4" max="12" width="7.875" customWidth="1"/>
     <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1499,13 +1499,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:13" ht="15.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:13" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="E8" s="58" t="s">
@@ -1520,7 +1520,7 @@
       <c r="L8" s="59"/>
       <c r="M8" s="60"/>
     </row>
-    <row r="9" spans="1:13" ht="105.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="29">
@@ -1559,43 +1559,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="55" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="25">
         <v>1241323</v>
       </c>
-      <c r="D10" s="53">
-        <v>5</v>
-      </c>
-      <c r="E10" s="26">
-        <v>5</v>
-      </c>
-      <c r="F10" s="27">
-        <v>5</v>
-      </c>
-      <c r="G10" s="27">
-        <v>4</v>
-      </c>
-      <c r="H10" s="27">
-        <v>4</v>
-      </c>
+      <c r="D10" s="53"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
       <c r="I10" s="27"/>
       <c r="J10" s="27"/>
       <c r="K10" s="25"/>
-      <c r="L10" s="35">
+      <c r="L10" s="35" t="e">
         <f t="shared" ref="L10:L17" si="0">AVERAGE(D10:K10)</f>
-        <v>4.5999999999999996</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="56"/>
       <c r="C11" s="6">
         <v>1241176</v>
       </c>
       <c r="D11" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11" s="53">
         <v>5</v>
@@ -1604,7 +1594,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H11" s="6">
         <v>4</v>
@@ -1614,10 +1604,10 @@
       <c r="K11" s="8"/>
       <c r="L11" s="36">
         <f t="shared" si="0"/>
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="56"/>
       <c r="C12" s="6">
         <v>1241166</v>
@@ -1645,7 +1635,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="56"/>
       <c r="C13" s="6">
         <v>1241285</v>
@@ -1673,13 +1663,13 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="56"/>
       <c r="C14" s="6">
         <v>1220804</v>
       </c>
       <c r="D14" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" s="6">
         <v>5</v>
@@ -1688,7 +1678,7 @@
         <v>5</v>
       </c>
       <c r="G14" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" s="53">
         <v>4</v>
@@ -1701,7 +1691,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="56"/>
       <c r="C15" s="6" t="s">
         <v>6</v>
@@ -1719,7 +1709,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="56"/>
       <c r="C16" s="6" t="s">
         <v>7</v>
@@ -1737,7 +1727,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="57"/>
       <c r="C17" s="28" t="s">
         <v>8</v>
@@ -1755,30 +1745,30 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="1"/>
       <c r="C18" s="32" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="33">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>4.4000000000000004</v>
+        <v>3.75</v>
       </c>
       <c r="E18" s="33">
         <f t="shared" si="1"/>
-        <v>4.5999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="F18" s="33">
         <f t="shared" si="1"/>
-        <v>4.8</v>
+        <v>4.75</v>
       </c>
       <c r="G18" s="33">
         <f t="shared" si="1"/>
-        <v>2.2000000000000002</v>
+        <v>2.5</v>
       </c>
       <c r="H18" s="33">
         <f t="shared" si="1"/>
-        <v>3.8</v>
+        <v>3.75</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -1794,7 +1784,7 @@
       </c>
       <c r="L18" s="38"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="42" t="s">
         <v>9</v>
       </c>
@@ -1810,7 +1800,7 @@
       <c r="K20" s="43"/>
       <c r="L20" s="44"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="45" t="s">
         <v>35</v>
       </c>
@@ -1826,7 +1816,7 @@
       <c r="K21" s="46"/>
       <c r="L21" s="47"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="48" t="s">
         <v>36</v>
       </c>
@@ -1842,7 +1832,7 @@
       <c r="K22" s="46"/>
       <c r="L22" s="47"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="45" t="s">
         <v>37</v>
       </c>
@@ -1858,7 +1848,7 @@
       <c r="K23" s="46"/>
       <c r="L23" s="47"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="45"/>
       <c r="B24" s="46"/>
       <c r="C24" s="46"/>
@@ -1872,7 +1862,7 @@
       <c r="K24" s="46"/>
       <c r="L24" s="47"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
         <v>38</v>
       </c>
@@ -1888,7 +1878,7 @@
       <c r="K25" s="46"/>
       <c r="L25" s="47"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="45">
         <v>0</v>
       </c>
@@ -1906,7 +1896,7 @@
       <c r="K26" s="46"/>
       <c r="L26" s="47"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="45">
         <v>1</v>
       </c>
@@ -1924,7 +1914,7 @@
       <c r="K27" s="46"/>
       <c r="L27" s="47"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="45">
         <v>2</v>
       </c>
@@ -1942,7 +1932,7 @@
       <c r="K28" s="46"/>
       <c r="L28" s="47"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="45">
         <v>3</v>
       </c>
@@ -1960,7 +1950,7 @@
       <c r="K29" s="46"/>
       <c r="L29" s="47"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="45">
         <v>4</v>
       </c>
@@ -1978,7 +1968,7 @@
       <c r="K30" s="46"/>
       <c r="L30" s="47"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="45">
         <v>5</v>
       </c>
@@ -1996,7 +1986,7 @@
       <c r="K31" s="46"/>
       <c r="L31" s="47"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="50"/>
       <c r="B32" s="51"/>
       <c r="C32" s="51"/>
@@ -2029,21 +2019,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="20.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="10" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="55" t="s">
         <v>17</v>
       </c>
@@ -2075,7 +2065,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="56"/>
       <c r="B4" s="64"/>
       <c r="C4" s="64"/>
@@ -2099,7 +2089,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="56"/>
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
@@ -2123,7 +2113,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>41</v>
       </c>
@@ -2153,7 +2143,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>42</v>
       </c>
@@ -2183,7 +2173,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>43</v>
       </c>
@@ -2213,7 +2203,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>44</v>
       </c>
@@ -2243,7 +2233,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>45</v>
       </c>
@@ -2273,7 +2263,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>46</v>
       </c>
@@ -2303,7 +2293,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>47</v>
       </c>
@@ -2333,7 +2323,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>48</v>
       </c>
@@ -2363,7 +2353,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>49</v>
       </c>
@@ -2393,7 +2383,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>50</v>
       </c>
@@ -2423,7 +2413,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>51</v>
       </c>
@@ -2453,7 +2443,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>52</v>
       </c>
@@ -2483,7 +2473,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>53</v>
       </c>
@@ -2515,7 +2505,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>54</v>
       </c>
@@ -2545,7 +2535,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>55</v>
       </c>
@@ -2575,7 +2565,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>56</v>
       </c>
@@ -2605,7 +2595,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>57</v>
       </c>
@@ -2635,7 +2625,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>58</v>
       </c>
@@ -2665,7 +2655,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>40</v>
       </c>
@@ -2695,7 +2685,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -2719,7 +2709,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -2743,7 +2733,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A27" s="11"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -2767,7 +2757,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A28" s="11"/>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -2791,7 +2781,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A29" s="11"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -2815,7 +2805,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A30" s="11"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -2839,7 +2829,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A31" s="11"/>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -2863,7 +2853,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="15"/>
       <c r="B32" s="39"/>
       <c r="C32" s="18"/>
@@ -2930,6 +2920,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3113,12 +3109,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
   <ds:schemaRefs>
@@ -3128,6 +3118,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3143,20 +3149,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
(docs): updated self assessment
</commit_message>
<xml_diff>
--- a/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint3/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcapa\IdeaProjects\sem2-pi24.25-G092-repo\docs\sprint3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63eef7978e99d393/Documents/GitHub/sem2-pi24.25-G092-repo/docs/sprint3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{9EAED4FF-FAA5-43AA-9C0C-1D1162579246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B95EE6A-C9EE-43F3-A4B1-60DE3849A320}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1095,7 +1095,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Instructions"/>
@@ -1464,33 +1464,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6.25" customWidth="1"/>
+    <col min="2" max="2" width="6.19921875" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="12" width="7.875" customWidth="1"/>
+    <col min="4" max="12" width="7.8984375" customWidth="1"/>
     <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1499,13 +1499,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:13" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:13" ht="15.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="E8" s="58" t="s">
@@ -1520,7 +1520,7 @@
       <c r="L8" s="59"/>
       <c r="M8" s="60"/>
     </row>
-    <row r="9" spans="1:13" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="105.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="29">
@@ -1559,27 +1559,37 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="55" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="25">
         <v>1241323</v>
       </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
+      <c r="D10" s="53">
+        <v>5</v>
+      </c>
+      <c r="E10" s="26">
+        <v>5</v>
+      </c>
+      <c r="F10" s="27">
+        <v>5</v>
+      </c>
+      <c r="G10" s="27">
+        <v>4</v>
+      </c>
+      <c r="H10" s="27">
+        <v>4</v>
+      </c>
       <c r="I10" s="27"/>
       <c r="J10" s="27"/>
       <c r="K10" s="25"/>
-      <c r="L10" s="35" t="e">
+      <c r="L10" s="35">
         <f t="shared" ref="L10:L17" si="0">AVERAGE(D10:K10)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="56"/>
       <c r="C11" s="6">
         <v>1241176</v>
@@ -1607,7 +1617,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="56"/>
       <c r="C12" s="6">
         <v>1241166</v>
@@ -1635,7 +1645,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="56"/>
       <c r="C13" s="6">
         <v>1241285</v>
@@ -1663,13 +1673,13 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="56"/>
       <c r="C14" s="6">
         <v>1220804</v>
       </c>
       <c r="D14" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" s="6">
         <v>5</v>
@@ -1678,20 +1688,20 @@
         <v>5</v>
       </c>
       <c r="G14" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I14" s="24"/>
       <c r="J14" s="6"/>
       <c r="K14" s="8"/>
       <c r="L14" s="36">
         <f t="shared" si="0"/>
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="56"/>
       <c r="C15" s="6" t="s">
         <v>6</v>
@@ -1709,7 +1719,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="56"/>
       <c r="C16" s="6" t="s">
         <v>7</v>
@@ -1727,7 +1737,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="57"/>
       <c r="C17" s="28" t="s">
         <v>8</v>
@@ -1745,30 +1755,30 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="1"/>
       <c r="C18" s="32" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="33">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
-        <v>3.75</v>
+        <v>4.2</v>
       </c>
       <c r="E18" s="33">
         <f t="shared" si="1"/>
-        <v>4.5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="F18" s="33">
         <f t="shared" si="1"/>
-        <v>4.75</v>
+        <v>4.8</v>
       </c>
       <c r="G18" s="33">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="H18" s="33">
         <f t="shared" si="1"/>
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="I18" s="33" t="e">
         <f t="shared" si="1"/>
@@ -1784,7 +1794,7 @@
       </c>
       <c r="L18" s="38"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="42" t="s">
         <v>9</v>
       </c>
@@ -1800,7 +1810,7 @@
       <c r="K20" s="43"/>
       <c r="L20" s="44"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="45" t="s">
         <v>35</v>
       </c>
@@ -1816,7 +1826,7 @@
       <c r="K21" s="46"/>
       <c r="L21" s="47"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="48" t="s">
         <v>36</v>
       </c>
@@ -1832,7 +1842,7 @@
       <c r="K22" s="46"/>
       <c r="L22" s="47"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="45" t="s">
         <v>37</v>
       </c>
@@ -1848,7 +1858,7 @@
       <c r="K23" s="46"/>
       <c r="L23" s="47"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="45"/>
       <c r="B24" s="46"/>
       <c r="C24" s="46"/>
@@ -1862,7 +1872,7 @@
       <c r="K24" s="46"/>
       <c r="L24" s="47"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="49" t="s">
         <v>38</v>
       </c>
@@ -1878,7 +1888,7 @@
       <c r="K25" s="46"/>
       <c r="L25" s="47"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="45">
         <v>0</v>
       </c>
@@ -1896,7 +1906,7 @@
       <c r="K26" s="46"/>
       <c r="L26" s="47"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="45">
         <v>1</v>
       </c>
@@ -1914,7 +1924,7 @@
       <c r="K27" s="46"/>
       <c r="L27" s="47"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="45">
         <v>2</v>
       </c>
@@ -1932,7 +1942,7 @@
       <c r="K28" s="46"/>
       <c r="L28" s="47"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="45">
         <v>3</v>
       </c>
@@ -1950,7 +1960,7 @@
       <c r="K29" s="46"/>
       <c r="L29" s="47"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="45">
         <v>4</v>
       </c>
@@ -1968,7 +1978,7 @@
       <c r="K30" s="46"/>
       <c r="L30" s="47"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="45">
         <v>5</v>
       </c>
@@ -1986,7 +1996,7 @@
       <c r="K31" s="46"/>
       <c r="L31" s="47"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="50"/>
       <c r="B32" s="51"/>
       <c r="C32" s="51"/>
@@ -2019,21 +2029,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="20.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.09765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="10" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="55" t="s">
         <v>17</v>
       </c>
@@ -2065,7 +2075,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A4" s="56"/>
       <c r="B4" s="64"/>
       <c r="C4" s="64"/>
@@ -2089,7 +2099,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="56"/>
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
@@ -2113,7 +2123,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>41</v>
       </c>
@@ -2143,7 +2153,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>42</v>
       </c>
@@ -2173,7 +2183,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>43</v>
       </c>
@@ -2203,7 +2213,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>44</v>
       </c>
@@ -2233,7 +2243,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>45</v>
       </c>
@@ -2263,7 +2273,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>46</v>
       </c>
@@ -2293,7 +2303,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>47</v>
       </c>
@@ -2323,7 +2333,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>48</v>
       </c>
@@ -2353,7 +2363,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>49</v>
       </c>
@@ -2383,7 +2393,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>50</v>
       </c>
@@ -2413,7 +2423,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>51</v>
       </c>
@@ -2443,7 +2453,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>52</v>
       </c>
@@ -2473,7 +2483,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>53</v>
       </c>
@@ -2505,7 +2515,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>54</v>
       </c>
@@ -2535,7 +2545,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>55</v>
       </c>
@@ -2565,7 +2575,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>56</v>
       </c>
@@ -2595,7 +2605,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>57</v>
       </c>
@@ -2625,7 +2635,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>58</v>
       </c>
@@ -2655,7 +2665,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>40</v>
       </c>
@@ -2685,7 +2695,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A25" s="11"/>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -2709,7 +2719,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A26" s="11"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -2733,7 +2743,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A27" s="11"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -2757,7 +2767,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A28" s="11"/>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -2781,7 +2791,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A29" s="11"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -2805,7 +2815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A30" s="11"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -2829,7 +2839,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A31" s="11"/>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -2853,7 +2863,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="15"/>
       <c r="B32" s="39"/>
       <c r="C32" s="18"/>
@@ -2920,12 +2930,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3109,6 +3113,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
   <ds:schemaRefs>
@@ -3118,22 +3128,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3149,4 +3143,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>